<commit_message>
adapté reporte de ventas de cuero para que ST 2 funcione bien en mayo 2026 que fue cuero y joyería. Completé proveedores. Descargué tax free del mayo. Faltan completar precios
</commit_message>
<xml_diff>
--- a/Codigo_paises.xlsx
+++ b/Codigo_paises.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="545">
   <si>
     <t>AFG</t>
   </si>
@@ -1653,6 +1653,12 @@
   </si>
   <si>
     <t>Congo</t>
+  </si>
+  <si>
+    <t>BOTC</t>
+  </si>
+  <si>
+    <t>Territorio Británico de Ultramar</t>
   </si>
 </sst>
 </file>
@@ -2083,7 +2089,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B274"/>
+  <dimension ref="A1:B275"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -4107,159 +4113,159 @@
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B253" s="2" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A254" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="B253" s="2" t="s">
+      <c r="B254" s="2" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="254" spans="1:2" ht="23" x14ac:dyDescent="0.35">
-      <c r="A254" s="1" t="s">
+    <row r="255" spans="1:2" ht="23" x14ac:dyDescent="0.35">
+      <c r="A255" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="B254" s="2" t="s">
+      <c r="B255" s="2" t="s">
         <v>495</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A255" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="B255" s="2" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>536</v>
+        <v>441</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>496</v>
+        <v>536</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>518</v>
+        <v>496</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>446</v>
+        <v>518</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>525</v>
+        <v>450</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>453</v>
+        <v>525</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>497</v>
+        <v>453</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>456</v>
+        <v>497</v>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>541</v>
+        <v>458</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B272" s="2" t="s">
         <v>541</v>
@@ -4267,17 +4273,25 @@
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>462</v>
+        <v>541</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="B274" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A275" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="B274" s="2" t="s">
+      <c r="B275" s="2" t="s">
         <v>464</v>
       </c>
     </row>

</xml_diff>